<commit_message>
feat: actualizar modulo bank-analyzer con reportes PDF uniformes, extractos bancarios y exportaciones
</commit_message>
<xml_diff>
--- a/_extractos/12.0 Respaldo bancario resumen de cuentas.xlsx
+++ b/_extractos/12.0 Respaldo bancario resumen de cuentas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOCUMENTOS\Contabilidad\Documentacion MAYAKI\Documentos Credito FIE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B68C58-3E19-4E7B-9160-F6C1AF2B47D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE647088-266D-4B72-9696-BCF2B34B1705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1100,11 +1100,11 @@
         <v>53</v>
       </c>
       <c r="G13" s="56">
-        <f>B13+B32+B51</f>
+        <f t="shared" ref="G13:H19" si="3">B13+B32+B51</f>
         <v>365882.59</v>
       </c>
       <c r="H13" s="56">
-        <f>C13+C32+C51</f>
+        <f t="shared" si="3"/>
         <v>318346.36000000004</v>
       </c>
     </row>
@@ -1126,11 +1126,11 @@
         <v>54</v>
       </c>
       <c r="G14" s="56">
-        <f>B14+B33+B52</f>
+        <f t="shared" si="3"/>
         <v>256510.88</v>
       </c>
       <c r="H14" s="56">
-        <f>C14+C33+C52</f>
+        <f t="shared" si="3"/>
         <v>240373.19</v>
       </c>
     </row>
@@ -1152,11 +1152,11 @@
         <v>55</v>
       </c>
       <c r="G15" s="56">
-        <f>B15+B34+B53</f>
+        <f t="shared" si="3"/>
         <v>124548.81000000001</v>
       </c>
       <c r="H15" s="56">
-        <f>C15+C34+C53</f>
+        <f t="shared" si="3"/>
         <v>188838.75</v>
       </c>
     </row>
@@ -1178,11 +1178,11 @@
         <v>56</v>
       </c>
       <c r="G16" s="56">
-        <f>B16+B35+B54</f>
+        <f t="shared" si="3"/>
         <v>76246.459999999992</v>
       </c>
       <c r="H16" s="56">
-        <f>C16+C35+C54</f>
+        <f t="shared" si="3"/>
         <v>73263.210000000006</v>
       </c>
     </row>
@@ -1204,11 +1204,11 @@
         <v>57</v>
       </c>
       <c r="G17" s="56">
-        <f>B17+B36+B55</f>
+        <f t="shared" si="3"/>
         <v>92165.75</v>
       </c>
       <c r="H17" s="56">
-        <f>C17+C36+C55</f>
+        <f t="shared" si="3"/>
         <v>96999.94</v>
       </c>
     </row>
@@ -1230,11 +1230,11 @@
         <v>58</v>
       </c>
       <c r="G18" s="56">
-        <f>B18+B37+B56</f>
+        <f t="shared" si="3"/>
         <v>57097.1</v>
       </c>
       <c r="H18" s="56">
-        <f>C18+C37+C56</f>
+        <f t="shared" si="3"/>
         <v>55545.39</v>
       </c>
     </row>
@@ -1256,22 +1256,22 @@
         <v>59</v>
       </c>
       <c r="G19" s="56">
-        <f>B19+B38+B57</f>
+        <f t="shared" si="3"/>
         <v>161489.38999999998</v>
       </c>
       <c r="H19" s="56">
-        <f>C19+C38+C57</f>
-        <v>155083.40000000002</v>
+        <f t="shared" si="3"/>
+        <v>155103.40000000002</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="34"/>
       <c r="B20" s="35">
-        <f t="shared" ref="B20:C20" si="3">SUM(B7:B19)</f>
+        <f t="shared" ref="B20:C20" si="4">SUM(B7:B19)</f>
         <v>1421694.27</v>
       </c>
       <c r="C20" s="35">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1418667.75</v>
       </c>
       <c r="D20" s="36"/>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="H20" s="56">
         <f>SUM(H7:H19)</f>
-        <v>1615115.1599999997</v>
+        <v>1615135.1599999997</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
@@ -1361,7 +1361,7 @@
         <v>1111.08</v>
       </c>
       <c r="D27" s="32">
-        <f t="shared" ref="D27:D38" si="4">D26+B27-C27</f>
+        <f t="shared" ref="D27:D38" si="5">D26+B27-C27</f>
         <v>545.85000000000014</v>
       </c>
       <c r="F27" s="24"/>
@@ -1377,7 +1377,7 @@
         <v>2075.6999999999998</v>
       </c>
       <c r="D28" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.1500000000005457</v>
       </c>
       <c r="F28" s="24"/>
@@ -1393,7 +1393,7 @@
         <v>330</v>
       </c>
       <c r="D29" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>120.15000000000055</v>
       </c>
       <c r="F29" s="24"/>
@@ -1409,7 +1409,7 @@
         <v>100</v>
       </c>
       <c r="D30" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>20.150000000000546</v>
       </c>
       <c r="F30" s="24"/>
@@ -1425,7 +1425,7 @@
         <v>8328.15</v>
       </c>
       <c r="D31" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>92.000000000001819</v>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
         <v>56626.400000000001</v>
       </c>
       <c r="D32" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>24987.599999999999</v>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
         <v>18224</v>
       </c>
       <c r="D33" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>29653.1</v>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         <v>33294.910000000003</v>
       </c>
       <c r="D34" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2978.1899999999951</v>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
         <v>5166.1099999999997</v>
       </c>
       <c r="D35" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>347.07999999999538</v>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
         <v>4888.0600000000004</v>
       </c>
       <c r="D36" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>19.01999999999498</v>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
         <v>1233.92</v>
       </c>
       <c r="D37" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>370.09999999999491</v>
       </c>
     </row>
@@ -1527,22 +1527,22 @@
         <v>300</v>
       </c>
       <c r="C38" s="33">
-        <v>350</v>
+        <v>370</v>
       </c>
       <c r="D38" s="32">
-        <f t="shared" si="4"/>
-        <v>320.09999999999491</v>
+        <f t="shared" si="5"/>
+        <v>300.09999999999491</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="37"/>
       <c r="B39" s="35">
-        <f t="shared" ref="B39:C39" si="5">SUM(B26:B38)</f>
+        <f t="shared" ref="B39:C39" si="6">SUM(B26:B38)</f>
         <v>130391.5</v>
       </c>
       <c r="C39" s="35">
-        <f t="shared" si="5"/>
-        <v>133187.63000000003</v>
+        <f t="shared" si="6"/>
+        <v>133207.63000000003</v>
       </c>
       <c r="D39" s="46"/>
     </row>
@@ -1637,7 +1637,7 @@
         <v>325.32</v>
       </c>
       <c r="D47" s="50">
-        <f t="shared" ref="D47:D57" si="6">D46+B47-C47</f>
+        <f t="shared" ref="D47:D57" si="7">D46+B47-C47</f>
         <v>140.23999999999995</v>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
         <v>0.03</v>
       </c>
       <c r="D48" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>140.42999999999995</v>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
         <v>480.02</v>
       </c>
       <c r="D49" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>72.169999999999959</v>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
         <v>0.01</v>
       </c>
       <c r="D50" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>72.269999999999953</v>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
         <v>4201.28</v>
       </c>
       <c r="D51" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>26955.08</v>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
         <v>15506.72</v>
       </c>
       <c r="D52" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>33057.31</v>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
         <v>33612.160000000003</v>
       </c>
       <c r="D53" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>104.63999999999214</v>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
         <v>0.08</v>
       </c>
       <c r="D54" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>707.86999999999205</v>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
         <v>4631.28</v>
       </c>
       <c r="D55" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>410.39999999999236</v>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
         <v>1489.15</v>
       </c>
       <c r="D56" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>38.819999999992206</v>
       </c>
     </row>
@@ -1787,7 +1787,7 @@
         <v>520.01</v>
       </c>
       <c r="D57" s="50">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>8.8599999999921693</v>
       </c>
     </row>
@@ -1825,7 +1825,7 @@
       <c r="B61" s="54"/>
       <c r="C61" s="35">
         <f>SUM(C13:C19)+SUM(C32:C38)+SUM(C51:C57)</f>
-        <v>1128450.24</v>
+        <v>1128470.24</v>
       </c>
       <c r="D61" s="46"/>
     </row>
@@ -1867,7 +1867,7 @@
       <c r="B66" s="54"/>
       <c r="C66" s="35">
         <f>C58+C39+C20</f>
-        <v>1615115.1600000001</v>
+        <v>1615135.1600000001</v>
       </c>
       <c r="D66" s="21"/>
     </row>

</xml_diff>